<commit_message>
add scaling method with hard bounds
</commit_message>
<xml_diff>
--- a/inst/templates/BMLMConfiguration.xlsx
+++ b/inst/templates/BMLMConfiguration.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="ParameterDefinition" sheetId="1" state="visible" r:id="rId3"/>
@@ -93,7 +93,7 @@
     <t xml:space="preserve">path of all linked parameter</t>
   </si>
   <si>
-    <t xml:space="preserve">if empty all secnarios,where parameter is defined</t>
+    <t xml:space="preserve">if empty all scenarios,where parameter is defined</t>
   </si>
   <si>
     <t xml:space="preserve">OutputPathId</t>
@@ -368,80 +368,84 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -782,12 +786,12 @@
   <mergeCells count="1">
     <mergeCell ref="F2:H2"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="6">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B3:B1002" type="list">
       <formula1>"global,individual"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I3:J1002" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I3:I1002" type="list">
       <formula1>"Linear,Log"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -797,6 +801,14 @@
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C3:C1002" type="list">
       <formula1>Dictionary!$B$2:$B$99</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J1:J2" type="none">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J3:J1002" type="list">
+      <formula1>"0,1"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -821,9 +833,9 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="30.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="7" width="30.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="7" width="14"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -875,7 +887,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.43359375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.15"/>
@@ -885,16 +897,16 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="8" t="s">
         <v>26</v>
       </c>
       <c r="E1" s="3" t="s">
@@ -920,8 +932,8 @@
       <formula1>Dictionary!$C$2:$C$9</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="A3:A1002" type="list">
-      <formula1>dictionary!#ref!</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:A1002" type="none">
+      <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -943,40 +955,40 @@
   <dimension ref="A1:S2"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="8" width="20.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="11.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="15.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="9" width="20.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="7" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="12.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="19.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="31.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="20.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="9" width="28.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="10" width="28.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="15" customFormat="true" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
+    <row r="1" s="16" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="14" t="s">
         <v>31</v>
       </c>
       <c r="I1" s="2" t="s">
@@ -985,31 +997,31 @@
       <c r="J1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="14" t="s">
+      <c r="L1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="10" t="s">
+      <c r="M1" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="N1" s="10" t="s">
+      <c r="N1" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="O1" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="P1" s="10" t="s">
+      <c r="P1" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="Q1" s="12" t="s">
+      <c r="Q1" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="R1" s="10" t="s">
+      <c r="R1" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="S1" s="12" t="s">
+      <c r="S1" s="13" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1023,14 +1035,14 @@
       <c r="C2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="17" t="s">
         <v>40</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
       <c r="H2" s="4" t="s">
         <v>13</v>
       </c>
@@ -1040,7 +1052,7 @@
       <c r="J2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="K2" s="16" t="s">
+      <c r="K2" s="17" t="s">
         <v>16</v>
       </c>
       <c r="L2" s="4" t="s">
@@ -1119,14 +1131,14 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="17.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="7" width="17.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="12.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="15.57"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
@@ -1138,13 +1150,13 @@
       <c r="D1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="14" t="s">
         <v>8</v>
       </c>
       <c r="H1" s="3" t="s">
@@ -1162,8 +1174,8 @@
       <c r="D2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
       <c r="G2" s="4" t="s">
         <v>16</v>
       </c>
@@ -1202,83 +1214,83 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="15.85"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="19" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="7" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="7" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="7" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="7" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="7" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="7" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="7" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="7" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="7" t="s">
         <v>68</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update vignette Overview graphic
</commit_message>
<xml_diff>
--- a/inst/templates/BMLMConfiguration.xlsx
+++ b/inst/templates/BMLMConfiguration.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="ParameterDefinition" sheetId="1" state="visible" r:id="rId3"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="71">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -120,6 +120,9 @@
     <t xml:space="preserve">HyperParameter</t>
   </si>
   <si>
+    <t xml:space="preserve">Final Value</t>
+  </si>
+  <si>
     <t xml:space="preserve">HyperDistribution</t>
   </si>
   <si>
@@ -151,6 +154,9 @@
   </si>
   <si>
     <t xml:space="preserve">if empty value is random</t>
+  </si>
+  <si>
+    <t xml:space="preserve">will be fille by export function</t>
   </si>
   <si>
     <t xml:space="preserve">for hyper parameter, this unit refers to individual start values</t>
@@ -928,12 +934,12 @@
     </row>
   </sheetData>
   <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:A1002" type="none">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B3:B1002" type="list">
       <formula1>Dictionary!$C$2:$C$9</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:A1002" type="none">
-      <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -952,18 +958,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="15.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="9" width="20.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="7" width="11.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="12.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="19.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="31.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="20.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="10" width="28.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="7" width="11.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="3" width="12.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="19.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="31.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="20.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="15.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="10" width="28.14"/>
   </cols>
   <sheetData>
     <row r="1" s="16" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -983,45 +989,48 @@
         <v>5</v>
       </c>
       <c r="F1" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="H1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="L1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="15" t="s">
+      <c r="M1" s="15" t="s">
         <v>2</v>
-      </c>
-      <c r="M1" s="11" t="s">
-        <v>32</v>
       </c>
       <c r="N1" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="P1" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="Q1" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="R1" s="11" t="s">
+      <c r="R1" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="S1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="T1" s="13" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1030,88 +1039,91 @@
         <v>20</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" s="18"/>
+        <v>42</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>43</v>
+      </c>
       <c r="G2" s="18"/>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="18"/>
+      <c r="I2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K2" s="17" t="s">
+      <c r="K2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L2" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="L2" s="4" t="s">
-        <v>43</v>
-      </c>
       <c r="M2" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="R2" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="S2" s="4"/>
+        <v>50</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="T2" s="4"/>
     </row>
   </sheetData>
   <dataValidations count="7">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" prompt="For logarithmic values use =LN(value)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="N1 P1 R1" type="none">
-      <formula1>0</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="K3:K1002" type="list">
-      <formula1>"Linear,Log"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I3:I1002" type="list">
-      <formula1>"1,0"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="A3:A1002" type="list">
       <formula1>ParameterDefinition!$A$2:$A$100</formula1>
       <formula2>0</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" prompt="For logarithmic values use =LN(value)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="O1 Q1 S1" type="none">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="L3:L1002" type="list">
+      <formula1>"Linear,Log"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="J3:J1002" type="list">
+      <formula1>"1,0"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B3:B1002" type="list">
       <formula1>Dictionary!$D$2:$D$19</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="L3:L1002" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="M3:M1002" type="list">
       <formula1>Dictionary!$B$2:$B$22</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="H3:H1002" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I3:I1002" type="list">
       <formula1>Dictionary!$B$3:$B$99</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" display="distribution for inividuals values (https://rdrr.io/r/stats/Distributions.html)"/>
-    <hyperlink ref="L2" r:id="rId2" display="https://rdrr.io/r/stats/Distributions.html&#10;"/>
+    <hyperlink ref="I2" r:id="rId1" display="distribution for inividuals values (https://rdrr.io/r/stats/Distributions.html)"/>
+    <hyperlink ref="M2" r:id="rId2" display="https://rdrr.io/r/stats/Distributions.html&#10;"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1128,13 +1140,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="7" width="17.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="11.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="12.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="15.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="7" width="11.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="12.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15.57"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1142,7 +1154,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>3</v>
@@ -1151,15 +1163,18 @@
         <v>5</v>
       </c>
       <c r="E1" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="G1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="H1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1168,18 +1183,21 @@
         <v>20</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E2" s="18"/>
+        <v>42</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>43</v>
+      </c>
       <c r="F2" s="18"/>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="18"/>
+      <c r="H2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -1187,7 +1205,7 @@
       <formula1>ParameterDefinition!$A$2:$A$100</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G3:G1002" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="H3:H1002" type="list">
       <formula1>"Linear,Log"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1219,7 +1237,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B1" s="19" t="s">
         <v>2</v>
@@ -1228,70 +1246,70 @@
         <v>24</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>